<commit_message>
fix: refine furniture grids and tabletop layering
</commit_message>
<xml_diff>
--- a/Excel/家具族表.xlsx
+++ b/Excel/家具族表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家具族" sheetId="1" r:id="R7164366536a845e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家具族" sheetId="1" r:id="Ra9dd193a329b4a91"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -535,20 +535,16 @@
           <x:t xml:space="preserve">table_lamp</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">台灯</x:t>
-        </x:is>
+      <x:c r="B3" t="str">
+        <x:v>经典落地灯</x:v>
       </x:c>
       <x:c r="C3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">灯具</x:t>
         </x:is>
       </x:c>
-      <x:c r="E3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E3" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F3" t="inlineStr">
         <x:is>
@@ -556,20 +552,18 @@
         </x:is>
       </x:c>
       <x:c r="G3" s="2" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H3" s="2" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">12</x:t>
         </x:is>
       </x:c>
-      <x:c r="J3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J3" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K3" t="inlineStr">
         <x:is>
@@ -603,20 +597,16 @@
           <x:t xml:space="preserve">round_table</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">圆桌</x:t>
-        </x:is>
+      <x:c r="B4" t="str">
+        <x:v>圆桌</x:v>
       </x:c>
       <x:c r="C4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E4" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F4" t="inlineStr">
         <x:is>
@@ -624,7 +614,7 @@
         </x:is>
       </x:c>
       <x:c r="G4" s="2" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H4" s="2" t="n">
         <x:v>5</x:v>
@@ -634,10 +624,8 @@
           <x:t xml:space="preserve">30</x:t>
         </x:is>
       </x:c>
-      <x:c r="J4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J4" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K4" t="inlineStr">
         <x:is>
@@ -650,19 +638,19 @@
         </x:is>
       </x:c>
       <x:c r="M4" s="2" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="N4" s="2" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="O4" s="2" t="n">
-        <x:v>20</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="P4" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q4" s="2" t="n">
-        <x:v>135</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -671,20 +659,16 @@
           <x:t xml:space="preserve">crescent_aquarium</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">月牙鱼缸</x:t>
-        </x:is>
+      <x:c r="B5" t="str">
+        <x:v>月牙鱼缸</x:v>
       </x:c>
       <x:c r="C5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E5" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F5" t="inlineStr">
         <x:is>
@@ -692,7 +676,7 @@
         </x:is>
       </x:c>
       <x:c r="G5" s="2" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H5" s="2" t="n">
         <x:v>1</x:v>
@@ -702,10 +686,8 @@
           <x:t xml:space="preserve">30</x:t>
         </x:is>
       </x:c>
-      <x:c r="J5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J5" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K5" t="inlineStr">
         <x:is>
@@ -739,20 +721,16 @@
           <x:t xml:space="preserve">cat_sofa</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">猫耳懒人沙发</x:t>
-        </x:is>
+      <x:c r="B6" t="str">
+        <x:v>猫耳懒人沙发</x:v>
       </x:c>
       <x:c r="C6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E6" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F6" t="inlineStr">
         <x:is>
@@ -760,7 +738,7 @@
         </x:is>
       </x:c>
       <x:c r="G6" s="2" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H6" s="2" t="n">
         <x:v>5</x:v>
@@ -770,10 +748,8 @@
           <x:t xml:space="preserve">25</x:t>
         </x:is>
       </x:c>
-      <x:c r="J6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J6" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K6" t="inlineStr">
         <x:is>
@@ -807,20 +783,16 @@
           <x:t xml:space="preserve">single_sofa</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">单人沙发</x:t>
-        </x:is>
+      <x:c r="B7" t="str">
+        <x:v>单人沙发</x:v>
       </x:c>
       <x:c r="C7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E7" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F7" t="inlineStr">
         <x:is>
@@ -828,7 +800,7 @@
         </x:is>
       </x:c>
       <x:c r="G7" s="2" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H7" s="2" t="n">
         <x:v>5</x:v>
@@ -838,10 +810,8 @@
           <x:t xml:space="preserve">32</x:t>
         </x:is>
       </x:c>
-      <x:c r="J7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J7" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K7" t="inlineStr">
         <x:is>
@@ -875,20 +845,16 @@
           <x:t xml:space="preserve">armchair</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">扶手椅</x:t>
-        </x:is>
+      <x:c r="B8" t="str">
+        <x:v>扶手椅</x:v>
       </x:c>
       <x:c r="C8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E8" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F8" t="inlineStr">
         <x:is>
@@ -896,7 +862,7 @@
         </x:is>
       </x:c>
       <x:c r="G8" s="2" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H8" s="2" t="n">
         <x:v>5</x:v>
@@ -906,10 +872,8 @@
           <x:t xml:space="preserve">30</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J8" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K8" t="inlineStr">
         <x:is>
@@ -943,20 +907,16 @@
           <x:t xml:space="preserve">cactus_lamp</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">仙人掌灯</x:t>
-        </x:is>
+      <x:c r="B9" t="str">
+        <x:v>仙人掌灯</x:v>
       </x:c>
       <x:c r="C9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">灯具</x:t>
         </x:is>
       </x:c>
-      <x:c r="E9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E9" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F9" t="inlineStr">
         <x:is>
@@ -974,10 +934,8 @@
           <x:t xml:space="preserve">15</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J9" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K9" t="inlineStr">
         <x:is>
@@ -1011,20 +969,16 @@
           <x:t xml:space="preserve">hanging_plant</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悬挂绿植</x:t>
-        </x:is>
+      <x:c r="B10" t="str">
+        <x:v>悬挂绿植</x:v>
       </x:c>
       <x:c r="C10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">盆栽</x:t>
         </x:is>
       </x:c>
-      <x:c r="E10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
+      <x:c r="E10" t="str">
+        <x:v>壁挂</x:v>
       </x:c>
       <x:c r="F10" t="inlineStr">
         <x:is>
@@ -1032,7 +986,7 @@
         </x:is>
       </x:c>
       <x:c r="G10" s="2" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H10" s="2" t="n">
         <x:v>7</x:v>
@@ -1042,10 +996,8 @@
           <x:t xml:space="preserve">18</x:t>
         </x:is>
       </x:c>
-      <x:c r="J10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J10" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K10" t="inlineStr">
         <x:is>
@@ -1079,20 +1031,16 @@
           <x:t xml:space="preserve">landscape_poster</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">风景海报</x:t>
-        </x:is>
+      <x:c r="B11" t="str">
+        <x:v>风景海报</x:v>
       </x:c>
       <x:c r="C11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">壁挂</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
+      <x:c r="E11" t="str">
+        <x:v>壁挂</x:v>
       </x:c>
       <x:c r="F11" t="inlineStr">
         <x:is>
@@ -1103,17 +1051,15 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="H11" s="2" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">15</x:t>
         </x:is>
       </x:c>
-      <x:c r="J11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J11" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K11" t="inlineStr">
         <x:is>
@@ -1147,20 +1093,16 @@
           <x:t xml:space="preserve">lava_lamp</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">熔岩灯</x:t>
-        </x:is>
+      <x:c r="B12" t="str">
+        <x:v>熔岩灯</x:v>
       </x:c>
       <x:c r="C12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">灯具</x:t>
         </x:is>
       </x:c>
-      <x:c r="E12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E12" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F12" t="inlineStr">
         <x:is>
@@ -1178,10 +1120,8 @@
           <x:t xml:space="preserve">15</x:t>
         </x:is>
       </x:c>
-      <x:c r="J12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J12" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K12" t="inlineStr">
         <x:is>
@@ -1215,20 +1155,16 @@
           <x:t xml:space="preserve">monstera</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">龟背竹</x:t>
-        </x:is>
+      <x:c r="B13" t="str">
+        <x:v>龟背竹</x:v>
       </x:c>
       <x:c r="C13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">盆栽</x:t>
         </x:is>
       </x:c>
-      <x:c r="E13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E13" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F13" t="inlineStr">
         <x:is>
@@ -1236,7 +1172,7 @@
         </x:is>
       </x:c>
       <x:c r="G13" s="2" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H13" s="2" t="n">
         <x:v>5</x:v>
@@ -1246,10 +1182,8 @@
           <x:t xml:space="preserve">20</x:t>
         </x:is>
       </x:c>
-      <x:c r="J13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J13" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K13" t="inlineStr">
         <x:is>
@@ -1283,20 +1217,16 @@
           <x:t xml:space="preserve">orb_decoration</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">球形摆件</x:t>
-        </x:is>
+      <x:c r="B14" t="str">
+        <x:v>球形摆件</x:v>
       </x:c>
       <x:c r="C14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E14" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F14" t="inlineStr">
         <x:is>
@@ -1304,7 +1234,7 @@
         </x:is>
       </x:c>
       <x:c r="G14" s="2" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H14" s="2" t="n">
         <x:v>1</x:v>
@@ -1314,10 +1244,8 @@
           <x:t xml:space="preserve">12</x:t>
         </x:is>
       </x:c>
-      <x:c r="J14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J14" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K14" t="inlineStr">
         <x:is>
@@ -1351,20 +1279,16 @@
           <x:t xml:space="preserve">potted_plant</x:t>
         </x:is>
       </x:c>
-      <x:c r="B15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">盆栽植物</x:t>
-        </x:is>
+      <x:c r="B15" t="str">
+        <x:v>盆栽植物</x:v>
       </x:c>
       <x:c r="C15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">盆栽</x:t>
         </x:is>
       </x:c>
-      <x:c r="E15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E15" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F15" t="inlineStr">
         <x:is>
@@ -1372,7 +1296,7 @@
         </x:is>
       </x:c>
       <x:c r="G15" s="2" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H15" s="2" t="n">
         <x:v>4</x:v>
@@ -1382,10 +1306,8 @@
           <x:t xml:space="preserve">12</x:t>
         </x:is>
       </x:c>
-      <x:c r="J15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J15" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K15" t="inlineStr">
         <x:is>
@@ -1419,20 +1341,16 @@
           <x:t xml:space="preserve">round_rug</x:t>
         </x:is>
       </x:c>
-      <x:c r="B16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">圆形地毯</x:t>
-        </x:is>
+      <x:c r="B16" t="str">
+        <x:v>圆形地毯</x:v>
       </x:c>
       <x:c r="C16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E16" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F16" t="inlineStr">
         <x:is>
@@ -1440,7 +1358,7 @@
         </x:is>
       </x:c>
       <x:c r="G16" s="2" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H16" s="2" t="n">
         <x:v>8</x:v>
@@ -1450,10 +1368,8 @@
           <x:t xml:space="preserve">15</x:t>
         </x:is>
       </x:c>
-      <x:c r="J16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J16" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K16" t="inlineStr">
         <x:is>
@@ -1487,20 +1403,16 @@
           <x:t xml:space="preserve">vintage_square_clock</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">复古方钟</x:t>
-        </x:is>
+      <x:c r="B17" t="str">
+        <x:v>复古方钟</x:v>
       </x:c>
       <x:c r="C17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">壁挂</x:t>
         </x:is>
       </x:c>
-      <x:c r="E17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
+      <x:c r="E17" t="str">
+        <x:v>壁挂</x:v>
       </x:c>
       <x:c r="F17" t="inlineStr">
         <x:is>
@@ -1508,7 +1420,7 @@
         </x:is>
       </x:c>
       <x:c r="G17" s="2" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H17" s="2" t="n">
         <x:v>5</x:v>
@@ -1518,10 +1430,8 @@
           <x:t xml:space="preserve">12</x:t>
         </x:is>
       </x:c>
-      <x:c r="J17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J17" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K17" t="inlineStr">
         <x:is>
@@ -1555,10 +1465,8 @@
           <x:t xml:space="preserve">bed_side</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">单人床</x:t>
-        </x:is>
+      <x:c r="B18" t="str">
+        <x:v>单人床</x:v>
       </x:c>
       <x:c r="C18" t="inlineStr">
         <x:is>
@@ -1570,10 +1478,8 @@
           <x:t xml:space="preserve">躺下去就不想起来的床。</x:t>
         </x:is>
       </x:c>
-      <x:c r="E18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E18" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F18" t="inlineStr">
         <x:is>
@@ -1591,10 +1497,8 @@
           <x:t xml:space="preserve">40</x:t>
         </x:is>
       </x:c>
-      <x:c r="J18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J18" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K18" t="inlineStr">
         <x:is>
@@ -1628,10 +1532,8 @@
           <x:t xml:space="preserve">bed_front</x:t>
         </x:is>
       </x:c>
-      <x:c r="B19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">床头床</x:t>
-        </x:is>
+      <x:c r="B19" t="str">
+        <x:v>床头床</x:v>
       </x:c>
       <x:c r="C19" t="inlineStr">
         <x:is>
@@ -1643,10 +1545,8 @@
           <x:t xml:space="preserve">床头是它的门面。</x:t>
         </x:is>
       </x:c>
-      <x:c r="E19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E19" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F19" t="inlineStr">
         <x:is>
@@ -1664,10 +1564,8 @@
           <x:t xml:space="preserve">40</x:t>
         </x:is>
       </x:c>
-      <x:c r="J19" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J19" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K19" t="inlineStr">
         <x:is>
@@ -1701,20 +1599,16 @@
           <x:t xml:space="preserve">vanity</x:t>
         </x:is>
       </x:c>
-      <x:c r="B20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">梳妆台</x:t>
-        </x:is>
+      <x:c r="B20" t="str">
+        <x:v>梳妆台</x:v>
       </x:c>
       <x:c r="C20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E20" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F20" t="inlineStr">
         <x:is>
@@ -1722,7 +1616,7 @@
         </x:is>
       </x:c>
       <x:c r="G20" s="2" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H20" s="2" t="n">
         <x:v>5</x:v>
@@ -1732,10 +1626,8 @@
           <x:t xml:space="preserve">35</x:t>
         </x:is>
       </x:c>
-      <x:c r="J20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J20" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K20" t="inlineStr">
         <x:is>
@@ -1769,20 +1661,16 @@
           <x:t xml:space="preserve">retro_radio</x:t>
         </x:is>
       </x:c>
-      <x:c r="B21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">复古收音机</x:t>
-        </x:is>
+      <x:c r="B21" t="str">
+        <x:v>复古收音机</x:v>
       </x:c>
       <x:c r="C21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E21" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F21" t="inlineStr">
         <x:is>
@@ -1800,10 +1688,8 @@
           <x:t xml:space="preserve">12</x:t>
         </x:is>
       </x:c>
-      <x:c r="J21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J21" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K21" t="inlineStr">
         <x:is>
@@ -1837,20 +1723,16 @@
           <x:t xml:space="preserve">music_player</x:t>
         </x:is>
       </x:c>
-      <x:c r="B22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">音乐播放器</x:t>
-        </x:is>
+      <x:c r="B22" t="str">
+        <x:v>音乐播放器</x:v>
       </x:c>
       <x:c r="C22" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E22" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F22" t="inlineStr">
         <x:is>
@@ -1858,7 +1740,7 @@
         </x:is>
       </x:c>
       <x:c r="G22" s="2" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H22" s="2" t="n">
         <x:v>5</x:v>
@@ -1868,10 +1750,8 @@
           <x:t xml:space="preserve">20</x:t>
         </x:is>
       </x:c>
-      <x:c r="J22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J22" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K22" t="inlineStr">
         <x:is>
@@ -1905,20 +1785,16 @@
           <x:t xml:space="preserve">piano</x:t>
         </x:is>
       </x:c>
-      <x:c r="B23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">钢琴</x:t>
-        </x:is>
+      <x:c r="B23" t="str">
+        <x:v>钢琴</x:v>
       </x:c>
       <x:c r="C23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E23" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F23" t="inlineStr">
         <x:is>
@@ -1926,7 +1802,7 @@
         </x:is>
       </x:c>
       <x:c r="G23" s="2" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H23" s="2" t="n">
         <x:v>7</x:v>
@@ -1936,10 +1812,8 @@
           <x:t xml:space="preserve">40</x:t>
         </x:is>
       </x:c>
-      <x:c r="J23" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J23" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K23" t="inlineStr">
         <x:is>
@@ -1973,20 +1847,16 @@
           <x:t xml:space="preserve">flashlight</x:t>
         </x:is>
       </x:c>
-      <x:c r="B24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">手电筒</x:t>
-        </x:is>
+      <x:c r="B24" t="str">
+        <x:v>手电筒</x:v>
       </x:c>
       <x:c r="C24" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E24" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F24" t="inlineStr">
         <x:is>
@@ -2004,10 +1874,8 @@
           <x:t xml:space="preserve">8</x:t>
         </x:is>
       </x:c>
-      <x:c r="J24" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J24" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K24" t="inlineStr">
         <x:is>
@@ -2041,20 +1909,16 @@
           <x:t xml:space="preserve">iron</x:t>
         </x:is>
       </x:c>
-      <x:c r="B25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">熨斗</x:t>
-        </x:is>
+      <x:c r="B25" t="str">
+        <x:v>熨斗</x:v>
       </x:c>
       <x:c r="C25" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E25" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F25" t="inlineStr">
         <x:is>
@@ -2072,10 +1936,8 @@
           <x:t xml:space="preserve">8</x:t>
         </x:is>
       </x:c>
-      <x:c r="J25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J25" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K25" t="inlineStr">
         <x:is>
@@ -2109,20 +1971,16 @@
           <x:t xml:space="preserve">telescope</x:t>
         </x:is>
       </x:c>
-      <x:c r="B26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">望远镜</x:t>
-        </x:is>
+      <x:c r="B26" t="str">
+        <x:v>望远镜</x:v>
       </x:c>
       <x:c r="C26" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E26" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F26" t="inlineStr">
         <x:is>
@@ -2130,7 +1988,7 @@
         </x:is>
       </x:c>
       <x:c r="G26" s="2" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H26" s="2" t="n">
         <x:v>1</x:v>
@@ -2140,10 +1998,8 @@
           <x:t xml:space="preserve">10</x:t>
         </x:is>
       </x:c>
-      <x:c r="J26" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J26" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K26" t="inlineStr">
         <x:is>
@@ -2177,20 +2033,16 @@
           <x:t xml:space="preserve">colorful_cabinet</x:t>
         </x:is>
       </x:c>
-      <x:c r="B27" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">彩色柜子</x:t>
-        </x:is>
+      <x:c r="B27" t="str">
+        <x:v>彩色柜子</x:v>
       </x:c>
       <x:c r="C27" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E27" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E27" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F27" t="inlineStr">
         <x:is>
@@ -2198,7 +2050,7 @@
         </x:is>
       </x:c>
       <x:c r="G27" s="2" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H27" s="2" t="n">
         <x:v>5</x:v>
@@ -2208,10 +2060,8 @@
           <x:t xml:space="preserve">28</x:t>
         </x:is>
       </x:c>
-      <x:c r="J27" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J27" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K27" t="inlineStr">
         <x:is>
@@ -2245,20 +2095,16 @@
           <x:t xml:space="preserve">floor_lamp</x:t>
         </x:is>
       </x:c>
-      <x:c r="B28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">落地灯</x:t>
-        </x:is>
+      <x:c r="B28" t="str">
+        <x:v>落地灯</x:v>
       </x:c>
       <x:c r="C28" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">灯具</x:t>
         </x:is>
       </x:c>
-      <x:c r="E28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E28" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F28" t="inlineStr">
         <x:is>
@@ -2276,10 +2122,8 @@
           <x:t xml:space="preserve">18</x:t>
         </x:is>
       </x:c>
-      <x:c r="J28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J28" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K28" t="inlineStr">
         <x:is>
@@ -2313,20 +2157,16 @@
           <x:t xml:space="preserve">chalkboard</x:t>
         </x:is>
       </x:c>
-      <x:c r="B29" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">黑板</x:t>
-        </x:is>
+      <x:c r="B29" t="str">
+        <x:v>黑板</x:v>
       </x:c>
       <x:c r="C29" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E29" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E29" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F29" t="inlineStr">
         <x:is>
@@ -2344,10 +2184,8 @@
           <x:t xml:space="preserve">15</x:t>
         </x:is>
       </x:c>
-      <x:c r="J29" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J29" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K29" t="inlineStr">
         <x:is>
@@ -2381,20 +2219,16 @@
           <x:t xml:space="preserve">macaron_sofa</x:t>
         </x:is>
       </x:c>
-      <x:c r="B30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">马卡龙沙发</x:t>
-        </x:is>
+      <x:c r="B30" t="str">
+        <x:v>马卡龙沙发</x:v>
       </x:c>
       <x:c r="C30" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">桌椅</x:t>
         </x:is>
       </x:c>
-      <x:c r="E30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
+      <x:c r="E30" t="str">
+        <x:v>地面</x:v>
       </x:c>
       <x:c r="F30" t="inlineStr">
         <x:is>
@@ -2402,7 +2236,7 @@
         </x:is>
       </x:c>
       <x:c r="G30" s="2" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H30" s="2" t="n">
         <x:v>5</x:v>
@@ -2412,10 +2246,8 @@
           <x:t xml:space="preserve">30</x:t>
         </x:is>
       </x:c>
-      <x:c r="J30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_1</x:t>
-        </x:is>
+      <x:c r="J30" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_1</x:v>
       </x:c>
       <x:c r="K30" t="inlineStr">
         <x:is>
@@ -2449,20 +2281,16 @@
           <x:t xml:space="preserve">metronome</x:t>
         </x:is>
       </x:c>
-      <x:c r="B31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">节拍器</x:t>
-        </x:is>
+      <x:c r="B31" t="str">
+        <x:v>节拍器</x:v>
       </x:c>
       <x:c r="C31" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">摆件</x:t>
         </x:is>
       </x:c>
-      <x:c r="E31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">桌面</x:t>
-        </x:is>
+      <x:c r="E31" t="str">
+        <x:v>桌面</x:v>
       </x:c>
       <x:c r="F31" t="inlineStr">
         <x:is>
@@ -2480,10 +2308,8 @@
           <x:t xml:space="preserve">10</x:t>
         </x:is>
       </x:c>
-      <x:c r="J31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SoundEffect/2_Pickup_260813_2</x:t>
-        </x:is>
+      <x:c r="J31" t="str">
+        <x:v>SoundEffect/2_Pickup_260813_2</x:v>
       </x:c>
       <x:c r="K31" t="inlineStr">
         <x:is>

</xml_diff>